<commit_message>
update dm-dependencies for GUM12
</commit_message>
<xml_diff>
--- a/_build/utils/dm-dependencies/resources/non_dm_rules.xlsx
+++ b/_build/utils/dm-dependencies/resources/non_dm_rules.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Uni\Corpora\GUM\github\_build\utils\dm-dependencies\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2D072FC-B2EB-4390-AF8C-A042526F7CB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88B40118-EC64-46ED-8D90-BA2F4E1970D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{BF4EFA19-1866-4339-A4F4-33A768915554}"/>
   </bookViews>
@@ -21,6 +21,9 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
@@ -1042,7 +1045,7 @@
     <t>(accurate|aggressive|amaze|amazing|attractive|awesome|awful|bad|beautiful|big|cathartic|cautionary|clean|clear|commendable|complicated|considerable|cool|correct|crazy|critical|cute|dark|decent|different|difficult|dreadful|easy|efficient|enough|essential|excellent|excited|exciting|false|fantastic|fine|frightful|froughtful|frustrate|fun|fundamental|funny|glad|goddamn|good|great|gross|happy|hard|heady|healthy|heartwarming|high|historic|honest|icky|ideal|important|inaccurate|incorrect|insane|interesting|large|legendary|likely|long|low|lucky|magnificent|militant|natural|necessary|needy|nice|normal|okay|peaceful|perfect|pleasant|possible|practical|pretty|proud|rare|real|realistic|reliable|remarkable|right|sad|safe|same|scared|scary|scenic|significant|simple|small|smart|solid|sorry|special|strange|strong|stun|stunned|stupid|sure|surpries|surprising|sweet|tame|tired|toxic|trash|tremendous|true|unbelievable|unlikely|unnatural|unpalatable|unprecedented|useful|valuable|versatile|violent|warm|weird|wild|wild|wonderful|worth|wrong)</t>
   </si>
   <si>
-    <t>$attrib_verb = (accept|acknowledge|add|admit|afraid|agree|announce|argue|ask|assert|assess|assume|assure|aware|believe|bet|call|care|certain|chant|check|claim|comment|complain|concern|conclude|confirm|contend|convince|cry|decide|declare|demonstrate|determine|disappoint|discover|discuss|doubt|dream|emphasize|ensure|establish|estimate|exclaim|expect|explain|express|feel|figure|find|forget|gather|glad|guarantee|guess|happy|hear|hold|hope|hypothesize|imagine|implore|imply|indicate|inform|know|learn|lie|maintain|mean|mention|mindful|mutter|note|notice|observe|pant|perceive|point|posit|pray|predict|presume|promise|propose|proud|prove|quote|quoth|re-iterate|read|realise|realize|reason|recall|recognize|recommend|reiterate|remark|remember|remind|repeat|reply|report|resent|reveal|rule|say|scream|see|shout|show|shriek|shrug|sing|snap|start|state|stunned|submit|suggest|summarize|suppose|sure|surprise|surprised|suspect|swear|tell|terrify|think|trust|tweet|understand|vlog|whisper|wish|witness|wonder|worry|write|be%like|go%say|keep%mind|bear%mind|make%sure)</t>
+    <t>$attrib_verb = (accept|acknowledge|add|admit|afraid|agree|announce|argue|ask|assert|assess|assume|assure|aware|believe|bet|call|care|certain|chant|check|claim|comment|complain|concern|conclude|confirm|consider|contend|convince|cry|decide|declare|demonstrate|determine|disappoint|discover|discuss|doubt|dream|emphasize|ensure|establish|estimate|exclaim|expect|explain|express|exult|feel|figure|find|forget|gather|glad|guarantee|guess|happy|hear|hold|hope|hypothesize|imagine|implore|imply|indicate|inform|know|learn|lie|maintain|mean|mention|mindful|mutter|note|notice|observe|pant|perceive|point|posit|pray|predict|presume|promise|propose|proud|prove|quote|quoth|re-iterate|read|realise|realize|reason|recall|recognize|recommend|reiterate|remark|remember|remind|repeat|reply|report|request|resent|reveal|rule|say|scream|see|shout|show|shriek|shrug|sing|snap|start|state|stunned|submit|suggest|summarize|suppose|sure|surprise|surprised|suspect|swear|tell|terrify|think|trust|tweet|understand|vlog|warn|whisper|wish|witness|wonder|worry|write|yell|be%like|go%say|keep%mind|bear%mind|make%sure)</t>
   </si>
 </sst>
 </file>

</xml_diff>